<commit_message>
Feat: Atualização nos custo do projeto
</commit_message>
<xml_diff>
--- a/Documentação/Custos do Projeto.xlsx
+++ b/Documentação/Custos do Projeto.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DTG-2025\Desktop\PROJETOS\Apex\Documentação\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DTG-2025\Desktop\Apex\Documentação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EDCFC83-BAAB-41FF-82EC-98D6B75FFA23}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C0D3275-2A7E-4A61-ADDF-C314F8B1413E}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -364,6 +364,7 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -421,7 +422,6 @@
     <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Moeda" xfId="1" builtinId="4"/>
@@ -747,24 +747,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="19" t="s">
+      <c r="A2" s="20" t="s">
         <v>39</v>
       </c>
-      <c r="B2" s="20"/>
-      <c r="C2" s="20"/>
-      <c r="D2" s="20"/>
-      <c r="E2" s="20"/>
-      <c r="F2" s="21"/>
+      <c r="B2" s="21"/>
+      <c r="C2" s="21"/>
+      <c r="D2" s="21"/>
+      <c r="E2" s="21"/>
+      <c r="F2" s="22"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
@@ -874,22 +874,22 @@
       <c r="A8" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B8" s="27">
+      <c r="B8" s="28">
         <f>SUM(F4:F7)</f>
         <v>334800</v>
       </c>
-      <c r="C8" s="28"/>
-      <c r="D8" s="28"/>
-      <c r="E8" s="28"/>
-      <c r="F8" s="29"/>
+      <c r="C8" s="29"/>
+      <c r="D8" s="29"/>
+      <c r="E8" s="29"/>
+      <c r="F8" s="30"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A10" s="23" t="s">
+      <c r="A10" s="24" t="s">
         <v>40</v>
       </c>
-      <c r="B10" s="23"/>
-      <c r="C10" s="23"/>
-      <c r="D10" s="23"/>
+      <c r="B10" s="24"/>
+      <c r="C10" s="24"/>
+      <c r="D10" s="24"/>
       <c r="E10" s="7"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
@@ -981,18 +981,18 @@
       <c r="A17" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B17" s="27">
+      <c r="B17" s="28">
         <f>SUM(D12:D16)</f>
         <v>48000</v>
       </c>
-      <c r="C17" s="28"/>
-      <c r="D17" s="29"/>
+      <c r="C17" s="29"/>
+      <c r="D17" s="30"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A19" s="22" t="s">
+      <c r="A19" s="23" t="s">
         <v>41</v>
       </c>
-      <c r="B19" s="22"/>
+      <c r="B19" s="23"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
@@ -1045,44 +1045,44 @@
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A27" s="24" t="s">
+      <c r="A27" s="25" t="s">
         <v>42</v>
       </c>
-      <c r="B27" s="25"/>
-      <c r="C27" s="26"/>
+      <c r="B27" s="26"/>
+      <c r="C27" s="27"/>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A28" s="16" t="s">
+      <c r="A28" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="B28" s="17"/>
+      <c r="B28" s="18"/>
       <c r="C28" s="10">
         <v>334800</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A29" s="16" t="s">
+      <c r="A29" s="17" t="s">
         <v>31</v>
       </c>
-      <c r="B29" s="17"/>
+      <c r="B29" s="18"/>
       <c r="C29" s="10">
         <v>48000</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A30" s="16" t="s">
+      <c r="A30" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="B30" s="17"/>
+      <c r="B30" s="18"/>
       <c r="C30" s="10">
         <v>16500</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A31" s="16" t="s">
+      <c r="A31" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="B31" s="17"/>
+      <c r="B31" s="18"/>
       <c r="C31" s="10">
         <f>SUM(C28:C30)</f>
         <v>399300</v>
@@ -1119,12 +1119,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="31" t="s">
         <v>43</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
+      <c r="B1" s="31"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
@@ -1208,19 +1208,19 @@
       <c r="A8" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="B8" s="27">
+      <c r="B8" s="28">
         <f>SUM(D4:D7)</f>
         <v>42000</v>
       </c>
-      <c r="C8" s="28"/>
-      <c r="D8" s="29"/>
+      <c r="C8" s="29"/>
+      <c r="D8" s="30"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A10" s="31" t="s">
+      <c r="A10" s="32" t="s">
         <v>45</v>
       </c>
-      <c r="B10" s="31"/>
-      <c r="C10" s="31"/>
+      <c r="B10" s="32"/>
+      <c r="C10" s="32"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
@@ -1270,18 +1270,18 @@
       <c r="A15" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="B15" s="27">
+      <c r="B15" s="28">
         <f>SUM(C12:C14)</f>
         <v>7500</v>
       </c>
-      <c r="C15" s="29"/>
+      <c r="C15" s="30"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A17" s="32" t="s">
+      <c r="A17" s="33" t="s">
         <v>44</v>
       </c>
-      <c r="B17" s="32"/>
-      <c r="C17" s="32"/>
+      <c r="B17" s="33"/>
+      <c r="C17" s="33"/>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="5" t="s">
@@ -1331,17 +1331,17 @@
       <c r="A22" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="B22" s="27">
+      <c r="B22" s="28">
         <f>SUM(C19:C21)</f>
         <v>9000</v>
       </c>
-      <c r="C22" s="29"/>
+      <c r="C22" s="30"/>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A24" s="33" t="s">
+      <c r="A24" s="34" t="s">
         <v>35</v>
       </c>
-      <c r="B24" s="34"/>
+      <c r="B24" s="35"/>
       <c r="C24" s="13"/>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
@@ -1362,8 +1362,8 @@
         <f>SUM(C12:C14)</f>
         <v>7500</v>
       </c>
-      <c r="E26" s="35"/>
-      <c r="F26" s="35"/>
+      <c r="E26" s="16"/>
+      <c r="F26" s="16"/>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" s="6" t="s">
@@ -1373,8 +1373,8 @@
         <f>SUM(C19:C21)</f>
         <v>9000</v>
       </c>
-      <c r="E27" s="35"/>
-      <c r="F27" s="35"/>
+      <c r="E27" s="16"/>
+      <c r="F27" s="16"/>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" s="6" t="s">
@@ -1384,40 +1384,40 @@
         <f>SUM(B25:B27)</f>
         <v>58500</v>
       </c>
-      <c r="E28" s="35"/>
-      <c r="F28" s="35"/>
+      <c r="E28" s="16"/>
+      <c r="F28" s="16"/>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E29" s="35"/>
-      <c r="F29" s="35"/>
+      <c r="E29" s="16"/>
+      <c r="F29" s="16"/>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E30" s="35"/>
-      <c r="F30" s="35"/>
+      <c r="E30" s="16"/>
+      <c r="F30" s="16"/>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E31" s="35"/>
-      <c r="F31" s="35"/>
+      <c r="E31" s="16"/>
+      <c r="F31" s="16"/>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E32" s="35"/>
-      <c r="F32" s="35"/>
+      <c r="E32" s="16"/>
+      <c r="F32" s="16"/>
     </row>
     <row r="33" spans="5:6" x14ac:dyDescent="0.3">
-      <c r="E33" s="35"/>
-      <c r="F33" s="35"/>
+      <c r="E33" s="16"/>
+      <c r="F33" s="16"/>
     </row>
     <row r="34" spans="5:6" x14ac:dyDescent="0.3">
-      <c r="E34" s="35"/>
-      <c r="F34" s="35"/>
+      <c r="E34" s="16"/>
+      <c r="F34" s="16"/>
     </row>
     <row r="35" spans="5:6" x14ac:dyDescent="0.3">
-      <c r="E35" s="35"/>
-      <c r="F35" s="35"/>
+      <c r="E35" s="16"/>
+      <c r="F35" s="16"/>
     </row>
     <row r="36" spans="5:6" x14ac:dyDescent="0.3">
-      <c r="E36" s="35"/>
-      <c r="F36" s="35"/>
+      <c r="E36" s="16"/>
+      <c r="F36" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="7">

</xml_diff>